<commit_message>
9. dispatch setting page chnages done and sample file
</commit_message>
<xml_diff>
--- a/rabbit-web-app/public/sample_excels/dispatch/carrier_bulk_sample.xlsx
+++ b/rabbit-web-app/public/sample_excels/dispatch/carrier_bulk_sample.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Carriers Bulk" sheetId="1" r:id="rId1"/>
+    <sheet name="Carriers" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,17 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
-  <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,22 +407,16 @@
         <v>address</v>
       </c>
       <c r="C1" t="str">
-        <v>mcNumber</v>
+        <v>primaryContact</v>
       </c>
       <c r="D1" t="str">
-        <v>dotNumber</v>
+        <v>email</v>
       </c>
       <c r="E1" t="str">
-        <v>primaryContact</v>
+        <v>cellPhone</v>
       </c>
       <c r="F1" t="str">
-        <v>email</v>
-      </c>
-      <c r="G1" t="str">
-        <v>phone</v>
-      </c>
-      <c r="H1" t="str">
-        <v>cellPhone</v>
+        <v>telephone</v>
       </c>
     </row>
     <row r="2">
@@ -443,22 +427,16 @@
         <v>Giriraj Annexe, Circuit House Road, Hubballi, Karnataka</v>
       </c>
       <c r="C2" t="str">
-        <v>MC-847291</v>
+        <v>Anand Sankeshwar</v>
       </c>
       <c r="D2" t="str">
-        <v>DOT-3920194</v>
+        <v>dispatch@vrllogistics.in</v>
       </c>
       <c r="E2" t="str">
-        <v>Anand Sankeshwar</v>
+        <v>94481 23456</v>
       </c>
       <c r="F2" t="str">
-        <v>dispatch@vrllogistics.in</v>
-      </c>
-      <c r="G2" t="str">
-        <v>+91 836 2237511</v>
-      </c>
-      <c r="H2" t="str">
-        <v>+91 94481 23456</v>
+        <v>836 2237511</v>
       </c>
     </row>
     <row r="3">
@@ -469,131 +447,101 @@
         <v>TCI House, 69 Institutional Area, Sector 32, Gurugram, Haryana</v>
       </c>
       <c r="C3" t="str">
-        <v>MC-918234</v>
+        <v>Vineet Agarwal</v>
       </c>
       <c r="D3" t="str">
-        <v>DOT-4102948</v>
+        <v>fleet@tcifreight.in</v>
       </c>
       <c r="E3" t="str">
-        <v>Vineet Agarwal</v>
+        <v>98112 34567</v>
       </c>
       <c r="F3" t="str">
-        <v>fleet@tcifreight.in</v>
-      </c>
-      <c r="G3" t="str">
-        <v>+91 124 2381603</v>
-      </c>
-      <c r="H3" t="str">
-        <v>+91 98112 34567</v>
+        <v>124 2381603</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Gati KWE Roadways</v>
+        <v>Gati-KWE Transport</v>
       </c>
       <c r="B4" t="str">
         <v>Plot No. 20, Western Hills, Kukatpally, Hyderabad, Telangana</v>
       </c>
       <c r="C4" t="str">
-        <v>MC-736251</v>
+        <v>Pirojshaw Sarkari</v>
       </c>
       <c r="D4" t="str">
-        <v>DOT-2839102</v>
+        <v>operations@gatikwe.com</v>
       </c>
       <c r="E4" t="str">
-        <v>Mahendra Agarwal</v>
+        <v>99490 12345</v>
       </c>
       <c r="F4" t="str">
-        <v>operations@gatikwe.com</v>
-      </c>
-      <c r="G4" t="str">
-        <v>+91 40 71204284</v>
-      </c>
-      <c r="H4" t="str">
-        <v>+91 99890 12345</v>
+        <v>40 27844284</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Safexpress Road Carriers</v>
+        <v>Safechem Logistics Fleet</v>
       </c>
       <c r="B5" t="str">
-        <v>Safex Cargo Complex, NH 8, Mahipalpur Extension, New Delhi</v>
+        <v>Safechem Complex, Sarkhej-Bavla Road, Ahmedabad, Gujarat</v>
       </c>
       <c r="C5" t="str">
-        <v>MC-625148</v>
+        <v>Mahesh Sharma</v>
       </c>
       <c r="D5" t="str">
-        <v>DOT-1928374</v>
+        <v>loads@safechemlogistics.com</v>
       </c>
       <c r="E5" t="str">
-        <v>Pawan Jain</v>
+        <v>98250 98765</v>
       </c>
       <c r="F5" t="str">
-        <v>contact@safexpress.com</v>
-      </c>
-      <c r="G5" t="str">
-        <v>+91 11 26783281</v>
-      </c>
-      <c r="H5" t="str">
-        <v>+91 98101 23456</v>
+        <v>79 26891023</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Allcargo Logistics Transport</v>
+        <v>Mahindra Logistics Transporters</v>
       </c>
       <c r="B6" t="str">
-        <v>Avvashya House, CST Road, Kalina, Santacruz East, Mumbai</v>
+        <v>1A &amp; 1B, Techniplex-I, Veer Savarkar Flyover, Goregaon West, Mumbai</v>
       </c>
       <c r="C6" t="str">
-        <v>MC-519284</v>
+        <v>Rampraveen Swaminathan</v>
       </c>
       <c r="D6" t="str">
-        <v>DOT-3847291</v>
+        <v>carriers@mahindralogistics.com</v>
       </c>
       <c r="E6" t="str">
-        <v>Shashi Kiran Shetty</v>
+        <v>98200 45678</v>
       </c>
       <c r="F6" t="str">
-        <v>dispatch@allcargologistics.com</v>
-      </c>
-      <c r="G6" t="str">
-        <v>+91 22 66798100</v>
-      </c>
-      <c r="H6" t="str">
-        <v>+91 98200 98765</v>
+        <v>22 28715500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Blue Dart Express Logistics</v>
+        <v>Delhivery Freight Line</v>
       </c>
       <c r="B7" t="str">
-        <v>Blue Dart Centre, Sahar Airport Road, Andheri East, Mumbai</v>
+        <v>Plot 5, Sector 44, Gurugram, Haryana</v>
       </c>
       <c r="C7" t="str">
-        <v>MC-410293</v>
+        <v>Sahil Barua</v>
       </c>
       <c r="D7" t="str">
-        <v>DOT-5928172</v>
+        <v>linehaul@delhivery.com</v>
       </c>
       <c r="E7" t="str">
-        <v>Balfour Manuel</v>
+        <v>98101 23456</v>
       </c>
       <c r="F7" t="str">
-        <v>carriers@bluedart.com</v>
-      </c>
-      <c r="G7" t="str">
-        <v>+91 22 28396444</v>
-      </c>
-      <c r="H7" t="str">
-        <v>+91 98210 54321</v>
+        <v>124 6719500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
37. Import carrier and manual add carrier dot and mc added
</commit_message>
<xml_diff>
--- a/rabbit-web-app/public/sample_excels/dispatch/carrier_bulk_sample.xlsx
+++ b/rabbit-web-app/public/sample_excels/dispatch/carrier_bulk_sample.xlsx
@@ -397,26 +397,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:H7"/>
+  <cols>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>name</v>
+        <v>Carrier Name</v>
       </c>
       <c r="B1" t="str">
-        <v>address</v>
+        <v>MC Number</v>
       </c>
       <c r="C1" t="str">
-        <v>primaryContact</v>
+        <v>DOT Number</v>
       </c>
       <c r="D1" t="str">
-        <v>email</v>
+        <v>Address</v>
       </c>
       <c r="E1" t="str">
-        <v>cellPhone</v>
+        <v>Primary Contact</v>
       </c>
       <c r="F1" t="str">
-        <v>telephone</v>
+        <v>Email</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Cell Phone</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Telephone</v>
       </c>
     </row>
     <row r="2">
@@ -424,18 +440,24 @@
         <v>VRL Logistics Ltd</v>
       </c>
       <c r="B2" t="str">
+        <v>874512</v>
+      </c>
+      <c r="C2" t="str">
+        <v>3498120</v>
+      </c>
+      <c r="D2" t="str">
         <v>Giriraj Annexe, Circuit House Road, Hubballi, Karnataka</v>
       </c>
-      <c r="C2" t="str">
+      <c r="E2" t="str">
         <v>Anand Sankeshwar</v>
       </c>
-      <c r="D2" t="str">
+      <c r="F2" t="str">
         <v>dispatch@vrllogistics.in</v>
       </c>
-      <c r="E2" t="str">
+      <c r="G2" t="str">
         <v>94481 23456</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>836 2237511</v>
       </c>
     </row>
@@ -444,18 +466,24 @@
         <v>TCI Freight Express</v>
       </c>
       <c r="B3" t="str">
+        <v>654321</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2987654</v>
+      </c>
+      <c r="D3" t="str">
         <v>TCI House, 69 Institutional Area, Sector 32, Gurugram, Haryana</v>
       </c>
-      <c r="C3" t="str">
+      <c r="E3" t="str">
         <v>Vineet Agarwal</v>
       </c>
-      <c r="D3" t="str">
+      <c r="F3" t="str">
         <v>fleet@tcifreight.in</v>
       </c>
-      <c r="E3" t="str">
+      <c r="G3" t="str">
         <v>98112 34567</v>
       </c>
-      <c r="F3" t="str">
+      <c r="H3" t="str">
         <v>124 2381603</v>
       </c>
     </row>
@@ -464,18 +492,24 @@
         <v>Gati-KWE Transport</v>
       </c>
       <c r="B4" t="str">
+        <v>543210</v>
+      </c>
+      <c r="C4" t="str">
+        <v>1876543</v>
+      </c>
+      <c r="D4" t="str">
         <v>Plot No. 20, Western Hills, Kukatpally, Hyderabad, Telangana</v>
       </c>
-      <c r="C4" t="str">
+      <c r="E4" t="str">
         <v>Pirojshaw Sarkari</v>
       </c>
-      <c r="D4" t="str">
+      <c r="F4" t="str">
         <v>operations@gatikwe.com</v>
       </c>
-      <c r="E4" t="str">
+      <c r="G4" t="str">
         <v>99490 12345</v>
       </c>
-      <c r="F4" t="str">
+      <c r="H4" t="str">
         <v>40 27844284</v>
       </c>
     </row>
@@ -484,18 +518,24 @@
         <v>Safechem Logistics Fleet</v>
       </c>
       <c r="B5" t="str">
+        <v>432109</v>
+      </c>
+      <c r="C5" t="str">
+        <v>4765432</v>
+      </c>
+      <c r="D5" t="str">
         <v>Safechem Complex, Sarkhej-Bavla Road, Ahmedabad, Gujarat</v>
       </c>
-      <c r="C5" t="str">
+      <c r="E5" t="str">
         <v>Mahesh Sharma</v>
       </c>
-      <c r="D5" t="str">
+      <c r="F5" t="str">
         <v>loads@safechemlogistics.com</v>
       </c>
-      <c r="E5" t="str">
+      <c r="G5" t="str">
         <v>98250 98765</v>
       </c>
-      <c r="F5" t="str">
+      <c r="H5" t="str">
         <v>79 26891023</v>
       </c>
     </row>
@@ -504,18 +544,24 @@
         <v>Mahindra Logistics Transporters</v>
       </c>
       <c r="B6" t="str">
+        <v>321098</v>
+      </c>
+      <c r="C6" t="str">
+        <v>3654321</v>
+      </c>
+      <c r="D6" t="str">
         <v>1A &amp; 1B, Techniplex-I, Veer Savarkar Flyover, Goregaon West, Mumbai</v>
       </c>
-      <c r="C6" t="str">
+      <c r="E6" t="str">
         <v>Rampraveen Swaminathan</v>
       </c>
-      <c r="D6" t="str">
+      <c r="F6" t="str">
         <v>carriers@mahindralogistics.com</v>
       </c>
-      <c r="E6" t="str">
+      <c r="G6" t="str">
         <v>98200 45678</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
         <v>22 28715500</v>
       </c>
     </row>
@@ -524,24 +570,30 @@
         <v>Delhivery Freight Line</v>
       </c>
       <c r="B7" t="str">
+        <v>210987</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2543210</v>
+      </c>
+      <c r="D7" t="str">
         <v>Plot 5, Sector 44, Gurugram, Haryana</v>
       </c>
-      <c r="C7" t="str">
+      <c r="E7" t="str">
         <v>Sahil Barua</v>
       </c>
-      <c r="D7" t="str">
+      <c r="F7" t="str">
         <v>linehaul@delhivery.com</v>
       </c>
-      <c r="E7" t="str">
+      <c r="G7" t="str">
         <v>98101 23456</v>
       </c>
-      <c r="F7" t="str">
+      <c r="H7" t="str">
         <v>124 6719500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>